<commit_message>
Update registry after gasoline prices fix
🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/data-registry.xlsx
+++ b/tools/data-registry.xlsx
@@ -449,7 +449,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3">
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X63"/>
+  <dimension ref="A1:X64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1405,17 +1405,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gdp-by-sector</t>
+          <t>exports-by-category</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mongolia GDP by Economic Sector (2024)</t>
+          <t>Mongolia Exports by Category, Thousands USD (1995-2024)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Монгол Улсын ДНБ эдийн засгийн салбараар (2024)</t>
+          <t>Монгол Улсын экспорт ангиллаар, мянган ам.доллар (1995-2024)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1423,55 +1423,39 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>nso-gdp-by-economic-activity</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Economy</t>
+          <t>Trade</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Эдийн засаг</t>
+          <t>Худалдаа</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>DT_NSO_1400_005V1_year.px</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/gdp-by-economic-activity.md</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>/datasets/gdp-by-sector-en.csv</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>content/data/en/gdp-by-sector.mdx</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>content/data/mn/gdp-by-sector.mdx</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>/charts/gdp-by-sector-en.json</t>
-        </is>
-      </c>
+          <t>sources/nso-1212/datasets/exports-by-category.md</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
@@ -1482,34 +1466,30 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>gdp-by-sector</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>2025-12-03 13:03:40</t>
-        </is>
-      </c>
+          <t>exports-by-category</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2025-12-05 02:38:00</t>
+          <t>2025-12-16 04:52:25</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>gdp-growth-rate</t>
+          <t>gdp-by-sector</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mongolia GDP Growth Rate (1991-2024)</t>
+          <t>Mongolia GDP by Economic Sector (2024)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Монгол Улсын ДНБ-ий өсөлтийн хувь (1991-2024)</t>
+          <t>Монгол Улсын ДНБ эдийн засгийн салбараар (2024)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1548,22 +1528,22 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>/datasets/gdp-growth-rate-en.csv</t>
+          <t>/datasets/gdp-by-sector-en.csv</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>content/data/en/gdp-growth-rate.mdx</t>
+          <t>content/data/en/gdp-by-sector.mdx</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>content/data/mn/gdp-growth-rate.mdx</t>
+          <t>content/data/mn/gdp-by-sector.mdx</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>/charts/gdp-growth-rate-en.json</t>
+          <t>/charts/gdp-by-sector-en.json</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1576,7 +1556,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>gdp-growth-rate</t>
+          <t>gdp-by-sector</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
@@ -1593,17 +1573,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>gdp-nominal</t>
+          <t>gdp-growth-rate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mongolia GDP at Current Prices (1990-2024)</t>
+          <t>Mongolia GDP Growth Rate (1991-2024)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Монгол Улсын ДНБ өнөөгийн үнээр (1990-2024)</t>
+          <t>Монгол Улсын ДНБ-ий өсөлтийн хувь (1991-2024)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1642,22 +1622,22 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>/datasets/gdp-nominal-en.csv</t>
+          <t>/datasets/gdp-growth-rate-en.csv</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>content/data/en/gdp-nominal.mdx</t>
+          <t>content/data/en/gdp-growth-rate.mdx</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>content/data/mn/gdp-nominal.mdx</t>
+          <t>content/data/mn/gdp-growth-rate.mdx</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>/charts/gdp-nominal-en.json</t>
+          <t>/charts/gdp-growth-rate-en.json</t>
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
@@ -1670,7 +1650,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>gdp-nominal</t>
+          <t>gdp-growth-rate</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1687,17 +1667,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gdp-real</t>
+          <t>gdp-nominal</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Mongolia Real GDP at 2015 Prices (1990-2024)</t>
+          <t>Mongolia GDP at Current Prices (1990-2024)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Монгол Улсын бодит ДНБ 2015 оны үнээр (1990-2024)</t>
+          <t>Монгол Улсын ДНБ өнөөгийн үнээр (1990-2024)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1736,22 +1716,22 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>/datasets/gdp-real-en.csv</t>
+          <t>/datasets/gdp-nominal-en.csv</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>content/data/en/gdp-real.mdx</t>
+          <t>content/data/en/gdp-nominal.mdx</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>content/data/mn/gdp-real.mdx</t>
+          <t>content/data/mn/gdp-nominal.mdx</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>/charts/gdp-real-en.json</t>
+          <t>/charts/gdp-nominal-en.json</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1764,7 +1744,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>gdp-real</t>
+          <t>gdp-nominal</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -1781,17 +1761,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gdp-sector-trends</t>
+          <t>gdp-real</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Mongolia GDP by Major Sectors Over Time (1990-2024)</t>
+          <t>Mongolia Real GDP at 2015 Prices (1990-2024)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Монгол Улсын ДНБ үндсэн салбаруудаар (1990-2024)</t>
+          <t>Монгол Улсын бодит ДНБ 2015 оны үнээр (1990-2024)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1825,27 +1805,27 @@
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/gdp-sector-trends.md</t>
+          <t>sources/nso-1212/datasets/gdp-by-economic-activity.md</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>/datasets/gdp-sector-trends-en.csv</t>
+          <t>/datasets/gdp-real-en.csv</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>content/data/en/gdp-sector-trends.mdx</t>
+          <t>content/data/en/gdp-real.mdx</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>content/data/mn/gdp-sector-trends.mdx</t>
+          <t>content/data/mn/gdp-real.mdx</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>/charts/gdp-sector-trends-en.json</t>
+          <t>/charts/gdp-real-en.json</t>
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
@@ -1858,7 +1838,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>gdp-sector-trends</t>
+          <t>gdp-real</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -1868,24 +1848,24 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2025-12-16 02:17:04</t>
+          <t>2025-12-05 02:38:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>gdp-usd</t>
+          <t>gdp-sector-trends</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Mongolia GDP in US Dollars (1990-2024)</t>
+          <t>Mongolia GDP by Major Sectors Over Time (1990-2024)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Монгол Улсын ДНБ ам.доллараар (1990-2024)</t>
+          <t>Монгол Улсын ДНБ үндсэн салбаруудаар (1990-2024)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1919,27 +1899,27 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/gdp-by-economic-activity.md</t>
+          <t>sources/nso-1212/datasets/gdp-sector-trends.md</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>/datasets/gdp-usd-en.csv</t>
+          <t>/datasets/gdp-sector-trends-en.csv</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>content/data/en/gdp-usd.mdx</t>
+          <t>content/data/en/gdp-sector-trends.mdx</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>content/data/mn/gdp-usd.mdx</t>
+          <t>content/data/mn/gdp-sector-trends.mdx</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>/charts/gdp-usd-en.json</t>
+          <t>/charts/gdp-sector-trends-en.json</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
@@ -1952,7 +1932,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>gdp-usd</t>
+          <t>gdp-sector-trends</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -1962,24 +1942,24 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2025-12-05 02:38:00</t>
+          <t>2025-12-16 02:17:04</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>household-income-by-location</t>
+          <t>gdp-usd</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Household Income: Urban vs Rural</t>
+          <t>Mongolia GDP in US Dollars (1990-2024)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Өрхийн орлого: Хот, хөдөө</t>
+          <t>Монгол Улсын ДНБ ам.доллараар (1990-2024)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1987,18 +1967,22 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>nso-gdp-by-economic-activity</t>
+        </is>
+      </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Household &amp; Income</t>
+          <t>Economy</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Өрх ба орлого</t>
+          <t>Эдийн засаг</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2009,13 +1993,29 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/household-income.md</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+          <t>sources/nso-1212/datasets/gdp-by-economic-activity.md</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>/datasets/gdp-usd-en.csv</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>content/data/en/gdp-usd.mdx</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>content/data/mn/gdp-usd.mdx</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>/charts/gdp-usd-en.json</t>
+        </is>
+      </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
@@ -2026,34 +2026,34 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>household-income-by-location</t>
+          <t>gdp-usd</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>2025-12-06T12:41:41.593565</t>
+          <t>2025-12-03 13:03:40</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2025-12-16 03:04:39</t>
+          <t>2025-12-05 02:38:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>household-income-total</t>
+          <t>household-income-by-location</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Mongolia Average Household Monthly Income</t>
+          <t>Household Income: Urban vs Rural</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Монгол Улсын өрхийн сарын дундаж орлого</t>
+          <t>Өрхийн орлого: Хот, хөдөө</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>household-income-total</t>
+          <t>household-income-by-location</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
@@ -2117,17 +2117,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>inflation-annual</t>
+          <t>household-income-total</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Mongolia Annual Inflation Rate (1991-2024)</t>
+          <t>Mongolia Average Household Monthly Income</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Монгол Улсын жилийн инфляцийн түвшин (1991-2024)</t>
+          <t>Монгол Улсын өрхийн сарын дундаж орлого</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2141,12 +2141,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Prices &amp; Inflation</t>
+          <t>Household &amp; Income</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Үнэ ба инфляци</t>
+          <t>Өрх ба орлого</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2154,12 +2154,12 @@
           <t>active</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>DT_NSO_0600_013V2.px</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>sources/nso-1212/datasets/household-income.md</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
@@ -2174,10 +2174,14 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>inflation-annual</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr"/>
+          <t>household-income-total</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>2025-12-06T12:41:41.593565</t>
+        </is>
+      </c>
       <c r="X19" t="inlineStr">
         <is>
           <t>2025-12-16 03:04:39</t>
@@ -2187,17 +2191,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>labor-participation-by-sex</t>
+          <t>inflation-annual</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Mongolia Labour Force Participation Rate by Sex (1992-2024)</t>
+          <t>Mongolia Annual Inflation Rate (1991-2024)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Монгол Улсын хөдөлмөрийн оролцооны түвшин хүйсээр (1992-2024)</t>
+          <t>Монгол Улсын жилийн инфляцийн түвшин (1991-2024)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2205,22 +2209,18 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>labor-participation-national</t>
-        </is>
-      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Labor Market</t>
+          <t>Prices &amp; Inflation</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Хөдөлмөрийн зах зээл</t>
+          <t>Үнэ ба инфляци</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2230,34 +2230,14 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>DT_NSO_0400_018V1_1.px</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>sources/nso-1212/datasets/labor-participation-by-sex.md</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>public/datasets/labor-participation-by-sex.csv</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>src/data/data/en/labor-participation-by-sex.mdx</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>src/data/data/mn/labor-participation-by-sex.mdx</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>public/charts/labor-participation-by-sex.json</t>
-        </is>
-      </c>
+          <t>DT_NSO_0600_013V2.px</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
@@ -2268,7 +2248,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>labor-participation-by-sex</t>
+          <t>inflation-annual</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -2281,27 +2261,31 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>labor-participation-by-sex</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mongolia Labour Force Participation Rate by Sex (1992-2024)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Монгол Улсын хөдөлмөрийн оролцооны түвшин хүйсээр (1992-2024)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>nso-1212</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>labor-participation-national</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Mongolia Labour Force Participation Rate (1992-2024)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Монгол Улсын хөдөлмөрийн оролцооны түвшин (1992-2024)</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>nso-1212</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -2325,27 +2309,27 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/labor-participation-national.md</t>
+          <t>sources/nso-1212/datasets/labor-participation-by-sex.md</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>public/datasets/labor-participation-national.csv</t>
+          <t>public/datasets/labor-participation-by-sex.csv</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>src/data/data/en/labor-participation-national.mdx</t>
+          <t>src/data/data/en/labor-participation-by-sex.mdx</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>src/data/data/mn/labor-participation-national.mdx</t>
+          <t>src/data/data/mn/labor-participation-by-sex.mdx</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>public/charts/labor-participation-national.json</t>
+          <t>public/charts/labor-participation-by-sex.json</t>
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
@@ -2358,7 +2342,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>labor-participation-national</t>
+          <t>labor-participation-by-sex</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -2371,17 +2355,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>livestock-by-type</t>
+          <t>labor-participation-national</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mongolia Livestock by Type (1970-2024)</t>
+          <t>Mongolia Labour Force Participation Rate (1992-2024)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Монгол Улсын мал төрлөөр (1970-2024)</t>
+          <t>Монгол Улсын хөдөлмөрийн оролцооны түвшин (1992-2024)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2389,22 +2373,18 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>livestock-total</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Agriculture</t>
+          <t>Labor Market</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Хөдөө аж ахуй</t>
+          <t>Хөдөлмөрийн зах зээл</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2414,18 +2394,34 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>DT_NSO_1001_109V1.px</t>
+          <t>DT_NSO_0400_018V1_1.px</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>tools/sources/nso-1212/datasets/livestock-by-type.md</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+          <t>sources/nso-1212/datasets/labor-participation-national.md</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>public/datasets/labor-participation-national.csv</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>src/data/data/en/labor-participation-national.mdx</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>src/data/data/mn/labor-participation-national.mdx</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>public/charts/labor-participation-national.json</t>
+        </is>
+      </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
@@ -2436,38 +2432,42 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>livestock-by-type</t>
+          <t>labor-participation-national</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2025-12-06 04:38:59</t>
+          <t>2025-12-16 03:04:39</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>livestock-by-type</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mongolia Livestock by Type (1970-2024)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Монгол Улсын мал төрлөөр (1970-2024)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>nso-1212</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>livestock-total</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Mongolia Total Livestock Count (1970-2024)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Монгол Улсын нийт малын тоо (1970-2024)</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>nso-1212</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
         <v>0</v>
       </c>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>tools/sources/nso-1212/datasets/livestock-total.md</t>
+          <t>tools/sources/nso-1212/datasets/livestock-by-type.md</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
@@ -2510,30 +2510,30 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>livestock-total</t>
+          <t>livestock-by-type</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2025-12-06 04:39:23</t>
+          <t>2025-12-06 04:38:59</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>nso-bop-monthly</t>
+          <t>livestock-total</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mongolia Balance of Payments (Monthly)</t>
+          <t>Mongolia Total Livestock Count (1970-2024)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Монгол Улсын төлбөрийн тэнцэл (Сараар)</t>
+          <t>Монгол Улсын нийт малын тоо (1970-2024)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2543,16 +2543,16 @@
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Economy</t>
+          <t>Agriculture</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Эдийн засаг</t>
+          <t>Хөдөө аж ахуй</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>DT_NSO_0100_001V10.px</t>
+          <t>DT_NSO_1001_109V1.px</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/bop-monthly.md</t>
+          <t>tools/sources/nso-1212/datasets/livestock-total.md</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
@@ -2580,30 +2580,34 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="n">
-        <v>0</v>
-      </c>
-      <c r="V24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>livestock-total</t>
+        </is>
+      </c>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2025-12-09 02:43:17</t>
+          <t>2025-12-06 04:39:23</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>nso-cpi-ulaanbaatar-mom</t>
+          <t>nso-bop-monthly</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CPI in Ulaanbaatar (Month-over-Month)</t>
+          <t>Mongolia Balance of Payments (Monthly)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Улаанбаатар хотын ХҮИ (Сар бүр)</t>
+          <t>Монгол Улсын төлбөрийн тэнцэл (Сараар)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2632,64 +2636,48 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DT_NSO_0600_003V4.px</t>
+          <t>DT_NSO_0100_001V10.px</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/nso-cpi-ulaanbaatar-mom.md</t>
+          <t>sources/nso-1212/datasets/bop-monthly.md</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>["Ulaanbaatar"]</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>city</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="n">
         <v>0</v>
       </c>
       <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr">
-        <is>
-          <t>2025-12-16T11:01:56.049093</t>
-        </is>
-      </c>
+      <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2025-12-16T11:01:56.049101</t>
+          <t>2025-12-09 02:43:17</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>nso-gdp-by-economic-activity</t>
+          <t>nso-cpi-ulaanbaatar-mom</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>GDP by Production Approach and Economic Activity</t>
+          <t>CPI in Ulaanbaatar (Month-over-Month)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ДНБ үйлдвэрлэлийн аргаар, эдийн засгийн салбараар</t>
+          <t>Улаанбаатар хотын ХҮИ (Сар бүр)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2718,26 +2706,34 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>DT_NSO_0500_001V1.px</t>
+          <t>DT_NSO_0600_003V4.px</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/gdp-by-economic-activity.md</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>versions/nso-gdp-by-economic-activity/</t>
-        </is>
-      </c>
+          <t>sources/nso-1212/datasets/nso-cpi-ulaanbaatar-mom.md</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>["Ulaanbaatar"]</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
       <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="n">
         <v>0</v>
@@ -2745,29 +2741,29 @@
       <c r="V26" t="inlineStr"/>
       <c r="W26" t="inlineStr">
         <is>
-          <t>2025-12-03 13:03:40</t>
+          <t>2025-12-16T11:01:56.049093</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2025-12-03 13:13:02</t>
+          <t>2025-12-16T11:01:56.049101</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>nso-population-age-sex</t>
+          <t>nso-gdp-by-economic-activity</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Population by Age Group and Sex</t>
+          <t>GDP by Production Approach and Economic Activity</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Хүн амын тоо насны бүлэг болон хүйсээр</t>
+          <t>ДНБ үйлдвэрлэлийн аргаар, эдийн засгийн салбараар</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2781,12 +2777,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Demographics</t>
+          <t>Economy</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Хүн ам зүй</t>
+          <t>Эдийн засаг</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2794,13 +2790,21 @@
           <t>active</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>DT_NSO_0500_001V1.px</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/nso-population-age-sex.md</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr"/>
+          <t>sources/nso-1212/datasets/gdp-by-economic-activity.md</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>versions/nso-gdp-by-economic-activity/</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
@@ -2815,29 +2819,29 @@
       <c r="V27" t="inlineStr"/>
       <c r="W27" t="inlineStr">
         <is>
-          <t>2025-12-05 01:51:21</t>
+          <t>2025-12-03 13:03:40</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2025-12-05 02:15:57</t>
+          <t>2025-12-03 13:13:02</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>nso-temperature-by-station</t>
+          <t>nso-population-age-sex</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Average Air Temperature by Station Location and Month</t>
+          <t>Population by Age Group and Sex</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Агаарын дундаж температур, станцын байршил, сараар</t>
+          <t>Хүн амын тоо насны бүлэг болон хүйсээр</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2851,12 +2855,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Demographics</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Байгаль орчин</t>
+          <t>Хүн ам зүй</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2864,14 +2868,10 @@
           <t>active</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>DT_NSO_2400_022V2.px</t>
-        </is>
-      </c>
+      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/temperature-by-station.md</t>
+          <t>sources/nso-1212/datasets/nso-population-age-sex.md</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
@@ -2887,23 +2887,31 @@
         <v>0</v>
       </c>
       <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>2025-12-05 01:51:21</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>2025-12-05 02:15:57</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>nso-unemployment-rate</t>
+          <t>nso-temperature-by-station</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Unemployment Rate by Category and Year</t>
+          <t>Average Air Temperature by Station Location and Month</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ажилгүйдлийн түвшин ангилал, жилээр</t>
+          <t>Агаарын дундаж температур, станцын байршил, сараар</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2917,12 +2925,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Labor Market</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Хөдөлмөрийн зах зээл</t>
+          <t>Байгаль орчин</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2932,12 +2940,12 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>DT_NSO_0400_049V1.px</t>
+          <t>DT_NSO_2400_022V2.px</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/unemployment-rate.md</t>
+          <t>sources/nso-1212/datasets/temperature-by-station.md</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
@@ -2959,17 +2967,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-aimags</t>
+          <t>nso-unemployment-rate</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Weekly Prices of Main Products (Aimags)</t>
+          <t>Unemployment Rate by Category and Year</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Үндсэн бүтээгдэхүүний долоо хоногийн үнэ (Аймгаар)</t>
+          <t>Ажилгүйдлийн түвшин ангилал, жилээр</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2983,12 +2991,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Economy</t>
+          <t>Labor Market</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Эдийн засаг</t>
+          <t>Хөдөлмөрийн зах зээл</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2998,68 +3006,44 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>DT_NSO_0300_010V5.px</t>
+          <t>DT_NSO_0400_049V1.px</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-prices-aimags.md</t>
+          <t>sources/nso-1212/datasets/unemployment-rate.md</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>["all_aimags", "regional_aggregates"]</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>aimag</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>2024-01</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>weekly</t>
-        </is>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>weekly-prices</t>
-        </is>
-      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
       <c r="U30" t="n">
         <v>0</v>
       </c>
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>2025-12-09 12:38:59</t>
-        </is>
-      </c>
+      <c r="X30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-ulaanbaatar</t>
+          <t>nso-weekly-prices-aimags</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Weekly Prices of Main Products and Gasoline (Ulaanbaatar)</t>
+          <t>Weekly Prices of Main Products (Aimags)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Үндсэн бүтээгдэхүүн, шатахууны долоо хоногийн үнэ (Улаанбаатар)</t>
+          <t>Үндсэн бүтээгдэхүүний долоо хоногийн үнэ (Аймгаар)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3073,12 +3057,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Prices &amp; Inflation</t>
+          <t>Economy</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Үнэ &amp; Инфляци</t>
+          <t>Эдийн засаг</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3088,12 +3072,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>DT_NSO_0600_001V4.px</t>
+          <t>DT_NSO_0300_010V5.px</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-prices-ulaanbaatar.md</t>
+          <t>sources/nso-1212/datasets/weekly-prices-aimags.md</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
@@ -3102,17 +3086,17 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>["Ulaanbaatar"]</t>
+          <t>["all_aimags", "regional_aggregates"]</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>aimag</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>2021-01-06</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3129,31 +3113,27 @@
         <v>0</v>
       </c>
       <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>2025-12-16T12:31:38.890823</t>
-        </is>
-      </c>
+      <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2025-12-16 04:35:54</t>
+          <t>2025-12-09 12:38:59</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>population-by-sex-mongolia</t>
+          <t>nso-weekly-prices-ulaanbaatar</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Population of Mongolia by Sex</t>
+          <t>Weekly Prices of Main Products and Gasoline (Ulaanbaatar)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Монгол Улсын хүн ам хүйсээр</t>
+          <t>Үндсэн бүтээгдэхүүн, шатахууны долоо хоногийн үнэ (Улаанбаатар)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3161,22 +3141,18 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>nso-population-age-sex</t>
-        </is>
-      </c>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Demographics</t>
+          <t>Prices &amp; Inflation</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Хүн ам зүй</t>
+          <t>Үнэ &amp; Инфляци</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3184,62 +3160,74 @@
           <t>active</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DT_NSO_0600_001V4.px</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/population-by-sex-mongolia.md</t>
+          <t>sources/nso-1212/datasets/weekly-prices-ulaanbaatar.md</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>src/data/data/en/population-by-sex-mongolia.mdx</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>src/data/data/mn/population-by-sex-mongolia.mdx</t>
-        </is>
-      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>["Ulaanbaatar"]</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>2021-01-06</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>weekly-prices</t>
+        </is>
+      </c>
       <c r="U32" t="n">
-        <v>1</v>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>population-by-sex-mongolia</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="V32" t="inlineStr"/>
       <c r="W32" t="inlineStr">
         <is>
-          <t>2025-12-05 01:51:21</t>
+          <t>2025-12-16T12:31:38.890823</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2025-12-05 02:38:00</t>
+          <t>2025-12-16 04:35:54</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>population-pyramid-mongolia</t>
+          <t>population-by-sex-mongolia</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Population Pyramid of Mongolia</t>
+          <t>Population of Mongolia by Sex</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Монгол Улсын хүн амын пирамид</t>
+          <t>Монгол Улсын хүн ам хүйсээр</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3273,18 +3261,18 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/population-pyramid-mongolia.md</t>
+          <t>sources/nso-1212/datasets/population-by-sex-mongolia.md</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr">
         <is>
-          <t>src/data/data/en/population-pyramid-mongolia.mdx</t>
+          <t>src/data/data/en/population-by-sex-mongolia.mdx</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>src/data/data/mn/population-pyramid-mongolia.mdx</t>
+          <t>src/data/data/mn/population-by-sex-mongolia.mdx</t>
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
@@ -3298,7 +3286,7 @@
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>population-pyramid-mongolia</t>
+          <t>population-by-sex-mongolia</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
@@ -3315,17 +3303,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>population-total-mongolia</t>
+          <t>population-pyramid-mongolia</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Total Population of Mongolia</t>
+          <t>Population Pyramid of Mongolia</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Монгол Улсын нийт хүн ам</t>
+          <t>Монгол Улсын хүн амын пирамид</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3359,18 +3347,18 @@
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/population-total-mongolia.md</t>
+          <t>sources/nso-1212/datasets/population-pyramid-mongolia.md</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
-          <t>src/data/data/en/population-total-mongolia.mdx</t>
+          <t>src/data/data/en/population-pyramid-mongolia.mdx</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>src/data/data/mn/population-total-mongolia.mdx</t>
+          <t>src/data/data/mn/population-pyramid-mongolia.mdx</t>
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
@@ -3384,7 +3372,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>population-total-mongolia</t>
+          <t>population-pyramid-mongolia</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
@@ -3394,24 +3382,24 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2025-12-05 02:53:07</t>
+          <t>2025-12-05 02:38:00</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>population-working-age-mongolia</t>
+          <t>population-total-mongolia</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Working Age Population of Mongolia (15-64)</t>
+          <t>Total Population of Mongolia</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Монгол Улсын ажиллах насны хүн ам (15-64)</t>
+          <t>Монгол Улсын нийт хүн ам</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3445,18 +3433,18 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/population-working-age-mongolia.md</t>
+          <t>sources/nso-1212/datasets/population-total-mongolia.md</t>
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
-          <t>src/data/data/en/population-working-age-mongolia.mdx</t>
+          <t>src/data/data/en/population-total-mongolia.mdx</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>src/data/data/mn/population-working-age-mongolia.mdx</t>
+          <t>src/data/data/mn/population-total-mongolia.mdx</t>
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
@@ -3470,7 +3458,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>population-working-age-mongolia</t>
+          <t>population-total-mongolia</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
@@ -3480,24 +3468,24 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2025-12-05 02:38:00</t>
+          <t>2025-12-05 02:53:07</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>salary-average-national</t>
+          <t>population-working-age-mongolia</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mongolia Average Monthly Salary (2001-2024)</t>
+          <t>Working Age Population of Mongolia (15-64)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Монгол Улсын сарын дундаж цалин (2001-2024)</t>
+          <t>Монгол Улсын ажиллах насны хүн ам (15-64)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3505,18 +3493,22 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>nso-population-age-sex</t>
+        </is>
+      </c>
       <c r="F36" t="n">
         <v>0</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Labor Market</t>
+          <t>Demographics</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Хөдөлмөрийн зах зээл</t>
+          <t>Хүн ам зүй</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3524,19 +3516,23 @@
           <t>active</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>DT_NSO_0400_022V1.px</t>
-        </is>
-      </c>
+      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>tools/sources/nso-1212/datasets/salary-average-national.md</t>
+          <t>sources/nso-1212/datasets/population-working-age-mongolia.md</t>
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>src/data/data/en/population-working-age-mongolia.mdx</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>src/data/data/mn/population-working-age-mongolia.mdx</t>
+        </is>
+      </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
@@ -3548,30 +3544,34 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>salary-average-national</t>
-        </is>
-      </c>
-      <c r="W36" t="inlineStr"/>
+          <t>population-working-age-mongolia</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>2025-12-05 01:51:21</t>
+        </is>
+      </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2025-12-16 03:04:39</t>
+          <t>2025-12-05 02:38:00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>salary-by-sector-2024</t>
+          <t>salary-average-national</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Average Monthly Salary by Economic Sector (2024)</t>
+          <t>Mongolia Average Monthly Salary (2001-2024)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Сарын дундаж цалин эдийн засгийн салбараар (2024)</t>
+          <t>Монгол Улсын сарын дундаж цалин (2001-2024)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3579,11 +3579,7 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>salary-average-national</t>
-        </is>
-      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="n">
         <v>0</v>
       </c>
@@ -3609,7 +3605,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>tools/sources/nso-1212/datasets/salary-by-sector-2024.md</t>
+          <t>tools/sources/nso-1212/datasets/salary-average-national.md</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
@@ -3626,7 +3622,7 @@
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>salary-by-sector-2024</t>
+          <t>salary-average-national</t>
         </is>
       </c>
       <c r="W37" t="inlineStr"/>
@@ -3639,17 +3635,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>temperature-anomaly</t>
+          <t>salary-by-sector-2024</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mongolia Temperature Anomaly vs 1981-2010 Baseline</t>
+          <t>Average Monthly Salary by Economic Sector (2024)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Монгол Улсын температурын хазайлт 1981-2010 суурь утгаас</t>
+          <t>Сарын дундаж цалин эдийн засгийн салбараар (2024)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3659,7 +3655,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>nso-temperature-by-station</t>
+          <t>salary-average-national</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -3667,12 +3663,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Environment</t>
+          <t>Labor Market</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Байгаль орчин</t>
+          <t>Хөдөлмөрийн зах зээл</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3682,12 +3678,12 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>DT_NSO_2400_022V2.px</t>
+          <t>DT_NSO_0400_022V1.px</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/temperature-by-station.md</t>
+          <t>tools/sources/nso-1212/datasets/salary-by-sector-2024.md</t>
         </is>
       </c>
       <c r="L38" t="inlineStr"/>
@@ -3700,26 +3696,34 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="n">
-        <v>0</v>
-      </c>
-      <c r="V38" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>salary-by-sector-2024</t>
+        </is>
+      </c>
       <c r="W38" t="inlineStr"/>
-      <c r="X38" t="inlineStr"/>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>2025-12-16 03:04:39</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>temperature-extremes-ulaanbaatar</t>
+          <t>temperature-anomaly</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Ulaanbaatar Temperature Extremes (2005-2025)</t>
+          <t>Mongolia Temperature Anomaly vs 1981-2010 Baseline</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Улаанбаатар хотын температурын хэт утга (2005-2025)</t>
+          <t>Монгол Улсын температурын хазайлт 1981-2010 суурь утгаас</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3779,17 +3783,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>temperature-regional</t>
+          <t>temperature-extremes-ulaanbaatar</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Mongolia Temperature by Region (2005-2025)</t>
+          <t>Ulaanbaatar Temperature Extremes (2005-2025)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Монгол Улсын температур бүс нутгаар (2005-2025)</t>
+          <t>Улаанбаатар хотын температурын хэт утга (2005-2025)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -3849,17 +3853,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>temperature-ulaanbaatar</t>
+          <t>temperature-regional</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ulaanbaatar Monthly Temperature (2005-2025)</t>
+          <t>Mongolia Temperature by Region (2005-2025)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Улаанбаатар хотын сарын дундаж температур (2005-2025)</t>
+          <t>Монгол Улсын температур бүс нутгаар (2005-2025)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3919,17 +3923,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>trade-exports-imports</t>
+          <t>temperature-ulaanbaatar</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mongolia Exports and Imports (1924-2024)</t>
+          <t>Ulaanbaatar Monthly Temperature (2005-2025)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Монгол Улсын экспорт, импорт (1924-2024)</t>
+          <t>Улаанбаатар хотын сарын дундаж температур (2005-2025)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3937,18 +3941,22 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>nso-temperature-by-station</t>
+        </is>
+      </c>
       <c r="F42" t="n">
         <v>0</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Trade</t>
+          <t>Environment</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Худалдаа</t>
+          <t>Байгаль орчин</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3956,10 +3964,14 @@
           <t>active</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>DT_NSO_2400_022V2.px</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>tools/sources/nso-1212/datasets/DT_NSO_1400_001V1_year.md</t>
+          <t>sources/nso-1212/datasets/temperature-by-station.md</t>
         </is>
       </c>
       <c r="L42" t="inlineStr"/>
@@ -3972,34 +3984,26 @@
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="n">
-        <v>1</v>
-      </c>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>trade-exports-imports</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="V42" t="inlineStr"/>
       <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr">
-        <is>
-          <t>2025-12-16 03:04:39</t>
-        </is>
-      </c>
+      <c r="X42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>trade-total</t>
+          <t>trade-exports-imports</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Mongolia Total Foreign Trade (1924-2024)</t>
+          <t>Mongolia Exports and Imports (1924-2024)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Монгол Улсын гадаад худалдааны нийт эргэлт (1924-2024)</t>
+          <t>Монгол Улсын экспорт, импорт (1924-2024)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4046,7 +4050,7 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>trade-total</t>
+          <t>trade-exports-imports</t>
         </is>
       </c>
       <c r="W43" t="inlineStr"/>
@@ -4059,17 +4063,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>unemployment-by-sex</t>
+          <t>trade-total</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Mongolia Unemployment Rate by Sex (2009-2024)</t>
+          <t>Mongolia Total Foreign Trade (1924-2024)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Монгол Улсын ажилгүйдлийн түвшин хүйсээр (2009-2024)</t>
+          <t>Монгол Улсын гадаад худалдааны нийт эргэлт (1924-2024)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -4077,22 +4081,18 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>unemployment-rate-national</t>
-        </is>
-      </c>
+      <c r="E44" t="inlineStr"/>
       <c r="F44" t="n">
         <v>0</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Labor Market</t>
+          <t>Trade</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Хөдөлмөрийн зах зээл</t>
+          <t>Худалдаа</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4100,14 +4100,10 @@
           <t>active</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>DT_NSO_0400_049V1.px</t>
-        </is>
-      </c>
+      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
-          <t>sources/nso-1212/DT_NSO_0400_049V1.px</t>
+          <t>tools/sources/nso-1212/datasets/DT_NSO_1400_001V1_year.md</t>
         </is>
       </c>
       <c r="L44" t="inlineStr"/>
@@ -4124,7 +4120,7 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>unemployment-by-sex</t>
+          <t>trade-total</t>
         </is>
       </c>
       <c r="W44" t="inlineStr"/>
@@ -4137,17 +4133,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>unemployment-rate-by-age</t>
+          <t>unemployment-by-sex</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Unemployment Rate by Age Group</t>
+          <t>Mongolia Unemployment Rate by Sex (2009-2024)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ажилгүйдлийн түвшин насны бүлгээр</t>
+          <t>Монгол Улсын ажилгүйдлийн түвшин хүйсээр (2009-2024)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4157,7 +4153,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>nso-unemployment-rate</t>
+          <t>unemployment-rate-national</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -4185,7 +4181,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/unemployment-rate.md</t>
+          <t>sources/nso-1212/DT_NSO_0400_049V1.px</t>
         </is>
       </c>
       <c r="L45" t="inlineStr"/>
@@ -4202,30 +4198,30 @@
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>unemployment-rate-by-age</t>
+          <t>unemployment-by-sex</t>
         </is>
       </c>
       <c r="W45" t="inlineStr"/>
       <c r="X45" t="inlineStr">
         <is>
-          <t>2025-12-07 06:56:47</t>
+          <t>2025-12-16 03:04:39</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>unemployment-rate-by-location</t>
+          <t>unemployment-rate-by-age</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Unemployment Rate by Location</t>
+          <t>Unemployment Rate by Age Group</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ажилгүйдлийн түвшин газар нутгаар</t>
+          <t>Ажилгүйдлийн түвшин насны бүлгээр</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -4280,7 +4276,7 @@
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>unemployment-rate-by-location</t>
+          <t>unemployment-rate-by-age</t>
         </is>
       </c>
       <c r="W46" t="inlineStr"/>
@@ -4293,17 +4289,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>unemployment-rate-by-region</t>
+          <t>unemployment-rate-by-location</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Unemployment Rate by Region</t>
+          <t>Unemployment Rate by Location</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Ажилгүйдлийн түвшин бүс нутгаар</t>
+          <t>Ажилгүйдлийн түвшин газар нутгаар</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4358,7 +4354,7 @@
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>unemployment-rate-by-region</t>
+          <t>unemployment-rate-by-location</t>
         </is>
       </c>
       <c r="W47" t="inlineStr"/>
@@ -4371,17 +4367,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>unemployment-rate-by-sex</t>
+          <t>unemployment-rate-by-region</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Unemployment Rate by Sex</t>
+          <t>Unemployment Rate by Region</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ажилгүйдлийн түвшин хүйсээр</t>
+          <t>Ажилгүйдлийн түвшин бүс нутгаар</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -4436,7 +4432,7 @@
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>unemployment-rate-by-sex</t>
+          <t>unemployment-rate-by-region</t>
         </is>
       </c>
       <c r="W48" t="inlineStr"/>
@@ -4449,17 +4445,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>unemployment-rate-national</t>
+          <t>unemployment-rate-by-sex</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Mongolia National Unemployment Rate (2009-2024)</t>
+          <t>Unemployment Rate by Sex</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Монгол Улсын ажилгүйдлийн түвшин (2009-2024)</t>
+          <t>Ажилгүйдлийн түвшин хүйсээр</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -4467,7 +4463,11 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>nso-unemployment-rate</t>
+        </is>
+      </c>
       <c r="F49" t="n">
         <v>0</v>
       </c>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>sources/nso-1212/DT_NSO_0400_049V1.px</t>
+          <t>sources/nso-1212/datasets/unemployment-rate.md</t>
         </is>
       </c>
       <c r="L49" t="inlineStr"/>
@@ -4510,30 +4510,30 @@
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>unemployment-rate-national</t>
+          <t>unemployment-rate-by-sex</t>
         </is>
       </c>
       <c r="W49" t="inlineStr"/>
       <c r="X49" t="inlineStr">
         <is>
-          <t>2025-12-16 03:04:39</t>
+          <t>2025-12-07 06:56:47</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>unemployment-rate-total</t>
+          <t>unemployment-rate-national</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Unemployment Rate of Mongolia</t>
+          <t>Mongolia National Unemployment Rate (2009-2024)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Монгол Улсын ажилгүйдлийн түвшин</t>
+          <t>Монгол Улсын ажилгүйдлийн түвшин (2009-2024)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -4541,11 +4541,7 @@
           <t>nso-1212</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>nso-unemployment-rate</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
       <c r="F50" t="n">
         <v>0</v>
       </c>
@@ -4571,7 +4567,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/unemployment-rate.md</t>
+          <t>sources/nso-1212/DT_NSO_0400_049V1.px</t>
         </is>
       </c>
       <c r="L50" t="inlineStr"/>
@@ -4588,30 +4584,30 @@
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>unemployment-rate-total</t>
+          <t>unemployment-rate-national</t>
         </is>
       </c>
       <c r="W50" t="inlineStr"/>
       <c r="X50" t="inlineStr">
         <is>
-          <t>2025-12-07 06:56:47</t>
+          <t>2025-12-16 03:04:39</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>unemployment-rate-youth</t>
+          <t>unemployment-rate-total</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Youth Unemployment Rate (15-24)</t>
+          <t>Unemployment Rate of Mongolia</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Залуучуудын ажилгүйдлийн түвшин (15-24)</t>
+          <t>Монгол Улсын ажилгүйдлийн түвшин</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4666,7 +4662,7 @@
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>unemployment-rate-youth</t>
+          <t>unemployment-rate-total</t>
         </is>
       </c>
       <c r="W51" t="inlineStr"/>
@@ -4679,17 +4675,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>weekly-beef-prices-aimags</t>
+          <t>unemployment-rate-youth</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Weekly Beef Prices by Region in Mongolia (2024-2025)</t>
+          <t>Youth Unemployment Rate (15-24)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Үхрийн махны долоо хоногийн үнэ, бүсээр (2024-2025)</t>
+          <t>Залуучуудын ажилгүйдлийн түвшин (15-24)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -4699,7 +4695,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-aimags</t>
+          <t>nso-unemployment-rate</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -4707,12 +4703,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Prices &amp; Inflation</t>
+          <t>Labor Market</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Үнэ ба инфляци</t>
+          <t>Хөдөлмөрийн зах зээл</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4720,66 +4716,54 @@
           <t>active</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>DT_NSO_0400_049V1.px</t>
+        </is>
+      </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-beef-prices-aimags.md</t>
+          <t>sources/nso-1212/datasets/unemployment-rate.md</t>
         </is>
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>["all_aimags", "regional_aggregates"]</t>
-        </is>
-      </c>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>aimag</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>2024-01</t>
-        </is>
-      </c>
-      <c r="S52" t="inlineStr">
-        <is>
-          <t>weekly</t>
-        </is>
-      </c>
-      <c r="T52" t="inlineStr">
-        <is>
-          <t>weekly-prices</t>
-        </is>
-      </c>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr"/>
       <c r="U52" t="n">
         <v>1</v>
       </c>
-      <c r="V52" t="inlineStr"/>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>unemployment-rate-youth</t>
+        </is>
+      </c>
       <c r="W52" t="inlineStr"/>
       <c r="X52" t="inlineStr">
         <is>
-          <t>2025-12-16 03:05:01</t>
+          <t>2025-12-07 06:56:47</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>weekly-bread-prices-ulaanbaatar</t>
+          <t>weekly-beef-prices-aimags</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Weekly Bread &amp; Grain Prices in Ulaanbaatar (2021-2025)</t>
+          <t>Weekly Beef Prices by Region in Mongolia (2024-2025)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Улаанбаатар дахь талх, гурилын бүтээгдэхүүний долоо хоногийн үнэ (2021-2025)</t>
+          <t>Үхрийн махны долоо хоногийн үнэ, бүсээр (2024-2025)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4789,7 +4773,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-ulaanbaatar</t>
+          <t>nso-weekly-prices-aimags</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -4802,7 +4786,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Үнэ &amp; Инфляци</t>
+          <t>Үнэ ба инфляци</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4813,42 +4797,26 @@
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-prices-ulaanbaatar.md</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>datasets/weekly-bread-prices-ulaanbaatar-en.csv</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>data/en/weekly-bread-prices-ulaanbaatar.mdx</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>data/mn/weekly-bread-prices-ulaanbaatar.mdx</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>charts/weekly-bread-prices-ulaanbaatar-en.json</t>
-        </is>
-      </c>
+          <t>sources/nso-1212/datasets/weekly-beef-prices-aimags.md</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
-          <t>["Ulaanbaatar"]</t>
+          <t>["all_aimags", "regional_aggregates"]</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>aimag</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>2021-01-06</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -4862,34 +4830,30 @@
         </is>
       </c>
       <c r="U53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr">
-        <is>
-          <t>2025-12-16T12:37:48.554103</t>
-        </is>
-      </c>
+      <c r="W53" t="inlineStr"/>
       <c r="X53" t="inlineStr">
         <is>
-          <t>2025-12-16T12:37:48.554103</t>
+          <t>2025-12-16 03:05:01</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>weekly-dairy-prices-ulaanbaatar</t>
+          <t>weekly-bread-prices-ulaanbaatar</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Weekly Dairy Prices in Ulaanbaatar (2021-2025)</t>
+          <t>Weekly Bread &amp; Grain Prices in Ulaanbaatar (2021-2025)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Улаанбаатар дахь сүү, сүүн бүтээгдэхүүний долоо хоногийн үнэ (2021-2025)</t>
+          <t>Улаанбаатар дахь талх, гурилын бүтээгдэхүүний долоо хоногийн үнэ (2021-2025)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -4928,22 +4892,22 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>datasets/weekly-dairy-prices-ulaanbaatar-en.csv</t>
+          <t>datasets/weekly-bread-prices-ulaanbaatar-en.csv</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>data/en/weekly-dairy-prices-ulaanbaatar.mdx</t>
+          <t>data/en/weekly-bread-prices-ulaanbaatar.mdx</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>data/mn/weekly-dairy-prices-ulaanbaatar.mdx</t>
+          <t>data/mn/weekly-bread-prices-ulaanbaatar.mdx</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>charts/weekly-dairy-prices-ulaanbaatar-en.json</t>
+          <t>charts/weekly-bread-prices-ulaanbaatar-en.json</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -4989,17 +4953,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>weekly-diesel-prices-aimags</t>
+          <t>weekly-dairy-prices-ulaanbaatar</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Weekly Diesel Prices by Region in Mongolia (2024-2025)</t>
+          <t>Weekly Dairy Prices in Ulaanbaatar (2021-2025)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Дизелийн түлшний долоо хоногийн үнэ, бүсээр (2024-2025)</t>
+          <t>Улаанбаатар дахь сүү, сүүн бүтээгдэхүүний долоо хоногийн үнэ (2021-2025)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -5009,7 +4973,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-aimags</t>
+          <t>nso-weekly-prices-ulaanbaatar</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -5022,7 +4986,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Үнэ ба инфляци</t>
+          <t>Үнэ &amp; Инфляци</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5033,26 +4997,42 @@
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-diesel-prices-aimags.md</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
+          <t>sources/nso-1212/datasets/weekly-prices-ulaanbaatar.md</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>datasets/weekly-dairy-prices-ulaanbaatar-en.csv</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>data/en/weekly-dairy-prices-ulaanbaatar.mdx</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>data/mn/weekly-dairy-prices-ulaanbaatar.mdx</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>charts/weekly-dairy-prices-ulaanbaatar-en.json</t>
+        </is>
+      </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>["all_aimags", "regional_aggregates"]</t>
+          <t>["Ulaanbaatar"]</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>aimag</t>
+          <t>city</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2021-01-06</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
@@ -5066,30 +5046,34 @@
         </is>
       </c>
       <c r="U55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V55" t="inlineStr"/>
-      <c r="W55" t="inlineStr"/>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>2025-12-16T12:37:48.554103</t>
+        </is>
+      </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>2025-12-16 03:05:01</t>
+          <t>2025-12-16T12:37:48.554103</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>weekly-flour-prices-aimags</t>
+          <t>weekly-diesel-prices-aimags</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Weekly Flour Prices by Region in Mongolia (2024-2025)</t>
+          <t>Weekly Diesel Prices by Region in Mongolia (2024-2025)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Гурилын долоо хоногийн үнэ, бүсээр (2024-2025)</t>
+          <t>Дизелийн түлшний долоо хоногийн үнэ, бүсээр (2024-2025)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -5123,7 +5107,7 @@
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-flour-prices-aimags.md</t>
+          <t>sources/nso-1212/datasets/weekly-diesel-prices-aimags.md</t>
         </is>
       </c>
       <c r="L56" t="inlineStr"/>
@@ -5169,17 +5153,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>weekly-fuel-prices-ulaanbaatar</t>
+          <t>weekly-flour-prices-aimags</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Weekly Fuel Prices in Ulaanbaatar (2021-2025)</t>
+          <t>Weekly Flour Prices by Region in Mongolia (2024-2025)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Улаанбаатар дахь шатахууны долоо хоногийн үнэ (2021-2025)</t>
+          <t>Гурилын долоо хоногийн үнэ, бүсээр (2024-2025)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -5189,7 +5173,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-ulaanbaatar</t>
+          <t>nso-weekly-prices-aimags</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -5202,7 +5186,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Үнэ &amp; Инфляци</t>
+          <t>Үнэ ба инфляци</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5213,42 +5197,26 @@
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-prices-ulaanbaatar.md</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>datasets/weekly-fuel-prices-ulaanbaatar-en.csv</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>data/en/weekly-fuel-prices-ulaanbaatar.mdx</t>
-        </is>
-      </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>data/mn/weekly-fuel-prices-ulaanbaatar.mdx</t>
-        </is>
-      </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>charts/weekly-fuel-prices-ulaanbaatar-en.json</t>
-        </is>
-      </c>
+          <t>sources/nso-1212/datasets/weekly-flour-prices-aimags.md</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
-          <t>["Ulaanbaatar"]</t>
+          <t>["all_aimags", "regional_aggregates"]</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>aimag</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>2021-01-06</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -5262,34 +5230,30 @@
         </is>
       </c>
       <c r="U57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V57" t="inlineStr"/>
-      <c r="W57" t="inlineStr">
-        <is>
-          <t>2025-12-16T12:37:48.554103</t>
-        </is>
-      </c>
+      <c r="W57" t="inlineStr"/>
       <c r="X57" t="inlineStr">
         <is>
-          <t>2025-12-16T12:37:48.554103</t>
+          <t>2025-12-16 03:05:01</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>weekly-gasoline-prices-aimags</t>
+          <t>weekly-fuel-prices-ulaanbaatar</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Weekly Gasoline (A-92) Prices by Region in Mongolia (2024-2025)</t>
+          <t>Weekly Fuel Prices in Ulaanbaatar (2021-2025)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Аи-92 автобензиний долоо хоногийн үнэ, бүсээр (2024-2025)</t>
+          <t>Улаанбаатар дахь шатахууны долоо хоногийн үнэ (2021-2025)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -5299,7 +5263,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-aimags</t>
+          <t>nso-weekly-prices-ulaanbaatar</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -5312,7 +5276,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Үнэ ба инфляци</t>
+          <t>Үнэ &amp; Инфляци</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5323,26 +5287,42 @@
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-prices-main-products.md</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
+          <t>sources/nso-1212/datasets/weekly-prices-ulaanbaatar.md</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>datasets/weekly-fuel-prices-ulaanbaatar-en.csv</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>data/en/weekly-fuel-prices-ulaanbaatar.mdx</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>data/mn/weekly-fuel-prices-ulaanbaatar.mdx</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>charts/weekly-fuel-prices-ulaanbaatar-en.json</t>
+        </is>
+      </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>["all_aimags", "regional_aggregates"]</t>
+          <t>["Ulaanbaatar"]</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>aimag</t>
+          <t>city</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2021-01-06</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
@@ -5356,30 +5336,34 @@
         </is>
       </c>
       <c r="U58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V58" t="inlineStr"/>
-      <c r="W58" t="inlineStr"/>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>2025-12-16T12:37:48.554103</t>
+        </is>
+      </c>
       <c r="X58" t="inlineStr">
         <is>
-          <t>2025-12-16 03:05:01</t>
+          <t>2025-12-16T12:37:48.554103</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>weekly-grocery-prices-ulaanbaatar</t>
+          <t>weekly-gasoline-prices-aimags</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Weekly Grocery Prices in Ulaanbaatar (2021-2025)</t>
+          <t>Weekly Gasoline (A-92) Prices by Region in Mongolia (2024-2025)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Улаанбаатар дахь хүнсний бүтээгдэхүүний долоо хоногийн үнэ (2021-2025)</t>
+          <t>Аи-92 автобензиний долоо хоногийн үнэ, бүсээр (2024-2025)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -5389,7 +5373,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-ulaanbaatar</t>
+          <t>nso-weekly-prices-aimags</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -5402,7 +5386,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Үнэ &amp; Инфляци</t>
+          <t>Үнэ ба инфляци</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5413,42 +5397,30 @@
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-prices-ulaanbaatar.md</t>
+          <t>sources/nso-1212/datasets/weekly-prices-main-products.md</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>datasets/weekly-grocery-prices-ulaanbaatar-en.csv</t>
-        </is>
-      </c>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>data/en/weekly-grocery-prices-ulaanbaatar.mdx</t>
-        </is>
-      </c>
-      <c r="N59" t="inlineStr">
-        <is>
-          <t>data/mn/weekly-grocery-prices-ulaanbaatar.mdx</t>
-        </is>
-      </c>
-      <c r="O59" t="inlineStr">
-        <is>
-          <t>charts/weekly-grocery-prices-ulaanbaatar-en.json</t>
-        </is>
-      </c>
+          <t>datasets/weekly-gasoline-prices-aimags-en.csv</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
-          <t>["Ulaanbaatar"]</t>
+          <t>["all_aimags", "regional_aggregates"]</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>aimag</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>2021-01-06</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -5462,34 +5434,30 @@
         </is>
       </c>
       <c r="U59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V59" t="inlineStr"/>
-      <c r="W59" t="inlineStr">
-        <is>
-          <t>2025-12-16T12:37:48.554103</t>
-        </is>
-      </c>
+      <c r="W59" t="inlineStr"/>
       <c r="X59" t="inlineStr">
         <is>
-          <t>2025-12-16T12:37:48.554103</t>
+          <t>2025-12-16 04:55:54</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>weekly-meat-prices-ulaanbaatar</t>
+          <t>weekly-grocery-prices-ulaanbaatar</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Weekly Meat Prices in Ulaanbaatar (2021-2025)</t>
+          <t>Weekly Grocery Prices in Ulaanbaatar (2021-2025)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Улаанбаатар дахь махны долоо хоногийн үнэ (2021-2025)</t>
+          <t>Улаанбаатар дахь хүнсний бүтээгдэхүүний долоо хоногийн үнэ (2021-2025)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -5528,22 +5496,22 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>datasets/weekly-meat-prices-ulaanbaatar-en.csv</t>
+          <t>datasets/weekly-grocery-prices-ulaanbaatar-en.csv</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>data/en/weekly-meat-prices-ulaanbaatar.mdx</t>
+          <t>data/en/weekly-grocery-prices-ulaanbaatar.mdx</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>data/mn/weekly-meat-prices-ulaanbaatar.mdx</t>
+          <t>data/mn/weekly-grocery-prices-ulaanbaatar.mdx</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>charts/weekly-meat-prices-ulaanbaatar-en.json</t>
+          <t>charts/weekly-grocery-prices-ulaanbaatar-en.json</t>
         </is>
       </c>
       <c r="P60" t="inlineStr">
@@ -5589,17 +5557,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>weekly-milk-prices-aimags</t>
+          <t>weekly-meat-prices-ulaanbaatar</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Weekly Fresh Milk Prices by Region in Mongolia (2024-2025)</t>
+          <t>Weekly Meat Prices in Ulaanbaatar (2021-2025)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Сүүний долоо хоногийн үнэ, бүсээр (2024-2025)</t>
+          <t>Улаанбаатар дахь махны долоо хоногийн үнэ (2021-2025)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -5609,7 +5577,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-aimags</t>
+          <t>nso-weekly-prices-ulaanbaatar</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -5622,7 +5590,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Үнэ ба инфляци</t>
+          <t>Үнэ &amp; Инфляци</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5633,26 +5601,42 @@
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr">
         <is>
-          <t>sources/nso-1212/datasets/weekly-prices-main-products.md</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
+          <t>sources/nso-1212/datasets/weekly-prices-ulaanbaatar.md</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>datasets/weekly-meat-prices-ulaanbaatar-en.csv</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>data/en/weekly-meat-prices-ulaanbaatar.mdx</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>data/mn/weekly-meat-prices-ulaanbaatar.mdx</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>charts/weekly-meat-prices-ulaanbaatar-en.json</t>
+        </is>
+      </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>["all_aimags", "regional_aggregates"]</t>
+          <t>["Ulaanbaatar"]</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>aimag</t>
+          <t>city</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2021-01-06</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -5666,30 +5650,34 @@
         </is>
       </c>
       <c r="U61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V61" t="inlineStr"/>
-      <c r="W61" t="inlineStr"/>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>2025-12-16T12:37:48.554103</t>
+        </is>
+      </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>2025-12-16 03:05:01</t>
+          <t>2025-12-16T12:37:48.554103</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>weekly-mutton-prices-aimags</t>
+          <t>weekly-milk-prices-aimags</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Weekly Mutton Prices by Region in Mongolia (2024-2025)</t>
+          <t>Weekly Fresh Milk Prices by Region in Mongolia (2024-2025)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Хонины махны долоо хоногийн үнэ, бүсээр (2024-2025)</t>
+          <t>Сүүний долоо хоногийн үнэ, бүсээр (2024-2025)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -5769,17 +5757,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>weekly-vegetable-prices-ulaanbaatar</t>
+          <t>weekly-mutton-prices-aimags</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Weekly Vegetable Prices in Ulaanbaatar (2021-2025)</t>
+          <t>Weekly Mutton Prices by Region in Mongolia (2024-2025)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Улаанбаатар дахь хүнсний ногооны долоо хоногийн үнэ (2021-2025)</t>
+          <t>Хонины махны долоо хоногийн үнэ, бүсээр (2024-2025)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -5789,7 +5777,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>nso-weekly-prices-ulaanbaatar</t>
+          <t>nso-weekly-prices-aimags</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -5802,7 +5790,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Үнэ &amp; Инфляци</t>
+          <t>Үнэ ба инфляци</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -5813,64 +5801,154 @@
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr">
         <is>
+          <t>sources/nso-1212/datasets/weekly-prices-main-products.md</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>["all_aimags", "regional_aggregates"]</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>aimag</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>weekly-prices</t>
+        </is>
+      </c>
+      <c r="U63" t="n">
+        <v>1</v>
+      </c>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr"/>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>2025-12-16 03:05:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>weekly-vegetable-prices-ulaanbaatar</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Weekly Vegetable Prices in Ulaanbaatar (2021-2025)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Улаанбаатар дахь хүнсний ногооны долоо хоногийн үнэ (2021-2025)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>nso-1212</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>nso-weekly-prices-ulaanbaatar</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Prices &amp; Inflation</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Үнэ &amp; Инфляци</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
           <t>sources/nso-1212/datasets/weekly-prices-ulaanbaatar.md</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr">
+      <c r="L64" t="inlineStr">
         <is>
           <t>datasets/weekly-vegetable-prices-ulaanbaatar-en.csv</t>
         </is>
       </c>
-      <c r="M63" t="inlineStr">
+      <c r="M64" t="inlineStr">
         <is>
           <t>data/en/weekly-vegetable-prices-ulaanbaatar.mdx</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr">
+      <c r="N64" t="inlineStr">
         <is>
           <t>data/mn/weekly-vegetable-prices-ulaanbaatar.mdx</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr">
+      <c r="O64" t="inlineStr">
         <is>
           <t>charts/weekly-vegetable-prices-ulaanbaatar-en.json</t>
         </is>
       </c>
-      <c r="P63" t="inlineStr">
+      <c r="P64" t="inlineStr">
         <is>
           <t>["Ulaanbaatar"]</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
+      <c r="Q64" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr">
+      <c r="R64" t="inlineStr">
         <is>
           <t>2021-01-06</t>
         </is>
       </c>
-      <c r="S63" t="inlineStr">
+      <c r="S64" t="inlineStr">
         <is>
           <t>weekly</t>
         </is>
       </c>
-      <c r="T63" t="inlineStr">
+      <c r="T64" t="inlineStr">
         <is>
           <t>weekly-prices</t>
         </is>
       </c>
-      <c r="U63" t="n">
-        <v>0</v>
-      </c>
-      <c r="V63" t="inlineStr"/>
-      <c r="W63" t="inlineStr">
+      <c r="U64" t="n">
+        <v>0</v>
+      </c>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr">
         <is>
           <t>2025-12-16T12:37:48.554103</t>
         </is>
       </c>
-      <c r="X63" t="inlineStr">
+      <c r="X64" t="inlineStr">
         <is>
           <t>2025-12-16T12:37:48.554103</t>
         </is>

</xml_diff>